<commit_message>
On branch master Changes to be committed: 	new file:   other/boot_keys.xlsx 	modified:   other/solar_and_battery_calculation.xlsx
</commit_message>
<xml_diff>
--- a/other/solar_and_battery_calculation.xlsx
+++ b/other/solar_and_battery_calculation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdul\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdul\Documents\gitFiles\cheatsheets\other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0B10E9-B173-45C7-9F24-B9309B6248DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB083436-2AF3-47CE-A231-3CB06B4F1023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>INVERTER BATTERY</t>
   </si>
@@ -73,12 +73,22 @@
   </si>
   <si>
     <t>EFFICIENCY (70%)</t>
+  </si>
+  <si>
+    <t>Select Cell, Ctrl+1, Number/Custom/Type[" Rs: "General]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="General&quot; AH&quot;"/>
+    <numFmt numFmtId="165" formatCode="General&quot; A&quot;"/>
+    <numFmt numFmtId="166" formatCode="General&quot; Hours&quot;"/>
+    <numFmt numFmtId="167" formatCode="General&quot; W&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot; Rs: &quot;General"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -108,8 +118,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -390,16 +405,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="39.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -407,15 +422,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>150</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -423,7 +438,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -431,17 +446,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <f>SUM(A2*70%)</f>
         <v>105</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <f>SUM(C2*80%)</f>
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -449,17 +464,17 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
         <f>SUM(A2/20)</f>
         <v>7.5</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="2">
         <f>SUM(C2/10)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -467,17 +482,17 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
         <f>SUM(A5/A7)</f>
         <v>14</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="3">
         <f>SUM(C5/C7)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -485,7 +500,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -493,17 +508,26 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
         <f>SUM(A7*22)</f>
         <v>165</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="4">
         <f>SUM(C7*22)</f>
         <v>330</v>
       </c>
+      <c r="F12" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>